<commit_message>
Updated AUS_grids_kan50 model - 2026-09-07 02:49
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
+++ b/VerveStacks_AUS_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
@@ -893,12 +893,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>e_Dubbo_AUS</t>
+          <t>e_MountPiper_AUS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>grid node -- way/169406848-330 (Central Coast, 226 km)</t>
+          <t>grid node -- way/169408193-330 (Sydney, 122 km)</t>
         </is>
       </c>
       <c r="D14" t="n">

</xml_diff>